<commit_message>
update code continue v1
</commit_message>
<xml_diff>
--- a/kinds_Listen_EPS.xlsx
+++ b/kinds_Listen_EPS.xlsx
@@ -1229,7 +1229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F262"/>
+  <dimension ref="A1:F265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2413,659 +2413,644 @@
         </is>
       </c>
     </row>
-    <row r="126" ht="22" customHeight="1">
-      <c r="A126" s="13" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>`trap_detail_distort`</t>
+        </is>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>Bóp méo chi tiết nhỏ trong nội dung</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>310002, 310003</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="6" t="inlineStr">
+        <is>
+          <t>`trap_action_swap`</t>
+        </is>
+      </c>
+      <c r="B126" s="6" t="inlineStr">
+        <is>
+          <t>Bức sai có đúng bối cảnh nhưng sai hành động</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="inlineStr">
+        <is>
+          <t>310003</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="6" t="inlineStr">
+        <is>
+          <t>`trap_context_swap`</t>
+        </is>
+      </c>
+      <c r="B127" s="6" t="inlineStr">
+        <is>
+          <t>Bức sai có đúng hành động nhưng sai bối cảnh</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="inlineStr">
+        <is>
+          <t>310003</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="22" customHeight="1">
+      <c r="A129" s="13" t="inlineStr">
         <is>
           <t>Quy tắc gán nhãn bẫy</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="11" t="inlineStr">
-        <is>
-          <t>• Mỗi câu hỏi có thể có NHIỀU nhãn bẫy cùng lúc</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="11" t="inlineStr">
-        <is>
-          <t>• Gán nhãn dựa trên ĐÁP ÁN SAI, không phải đáp án đúng</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="11" t="inlineStr">
-        <is>
-          <t>• Chỉ gán khi có bằng chứng rõ ràng, không suy đoán</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="11" t="inlineStr">
         <is>
+          <t>• Mỗi câu hỏi có thể có NHIỀU nhãn bẫy cùng lúc</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="11" t="inlineStr">
+        <is>
+          <t>• Gán nhãn dựa trên ĐÁP ÁN SAI, không phải đáp án đúng</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="11" t="inlineStr">
+        <is>
+          <t>• Chỉ gán khi có bằng chứng rõ ràng, không suy đoán</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="11" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="131" ht="22" customHeight="1">
-      <c r="A131" s="9" t="inlineStr">
+    <row r="134" ht="22" customHeight="1">
+      <c r="A134" s="9" t="inlineStr">
         <is>
           <t>Đặc điểm câu hỏi (question_feature)</t>
         </is>
       </c>
-      <c r="B131" s="10" t="n"/>
-      <c r="C131" s="10" t="n"/>
-      <c r="D131" s="10" t="n"/>
-      <c r="E131" s="10" t="n"/>
-      <c r="F131" s="10" t="n"/>
-    </row>
-    <row r="132" ht="22" customHeight="1">
-      <c r="A132" s="13" t="inlineStr">
+      <c r="B134" s="10" t="n"/>
+      <c r="C134" s="10" t="n"/>
+      <c r="D134" s="10" t="n"/>
+      <c r="E134" s="10" t="n"/>
+      <c r="F134" s="10" t="n"/>
+    </row>
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="13" t="inlineStr">
         <is>
           <t>Nhóm câu hỏi có q_text</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="14" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="14" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B133" s="14" t="inlineStr">
+      <c r="B136" s="14" t="inlineStr">
         <is>
           <t>Nhãn tiếng Anh</t>
         </is>
       </c>
-      <c r="C133" s="14" t="inlineStr">
+      <c r="C136" s="14" t="inlineStr">
         <is>
           <t>Mô tả</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="6" t="inlineStr">
-        <is>
-          <t>`qf_content_match`</t>
-        </is>
-      </c>
-      <c r="B134" s="6" t="inlineStr">
-        <is>
-          <t>Content Match</t>
-        </is>
-      </c>
-      <c r="C134" s="6" t="inlineStr">
-        <is>
-          <t>"들은 내용으로 맞는 것을 고르십시오"</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="6" t="inlineStr">
-        <is>
-          <t>`qf_what`</t>
-        </is>
-      </c>
-      <c r="B135" s="6" t="inlineStr">
-        <is>
-          <t>What (General)</t>
-        </is>
-      </c>
-      <c r="C135" s="6" t="inlineStr">
-        <is>
-          <t>"무엇입니까?", "무엇을 삽니까?"</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="6" t="inlineStr">
-        <is>
-          <t>`qf_what_doing`</t>
-        </is>
-      </c>
-      <c r="B136" s="6" t="inlineStr">
-        <is>
-          <t>What Doing</t>
-        </is>
-      </c>
-      <c r="C136" s="6" t="inlineStr">
-        <is>
-          <t>"무엇을 하고 있습니까?"</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>`qf_where`</t>
+          <t>`qf_content_match`</t>
         </is>
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
-          <t>Where/Which</t>
+          <t>Content Match</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">
         <is>
-          <t>"어디입니까?", "어느 나라?"</t>
+          <t>"들은 내용으로 맞는 것을 고르십시오"</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>`qf_central_thought`</t>
+          <t>`qf_what`</t>
         </is>
       </c>
       <c r="B138" s="6" t="inlineStr">
         <is>
-          <t>Central Thought</t>
+          <t>What (General)</t>
         </is>
       </c>
       <c r="C138" s="6" t="inlineStr">
         <is>
-          <t>"중심 생각으로 맞는 것"</t>
+          <t>"무엇입니까?", "무엇을 삽니까?"</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>`qf_why`</t>
+          <t>`qf_what_doing`</t>
         </is>
       </c>
       <c r="B139" s="6" t="inlineStr">
         <is>
-          <t>Why/Reason</t>
+          <t>What Doing</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>"왜?", "이유"</t>
+          <t>"무엇을 하고 있습니까?"</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>`qf_when_time`</t>
+          <t>`qf_where`</t>
         </is>
       </c>
       <c r="B140" s="6" t="inlineStr">
         <is>
-          <t>When/Time</t>
+          <t>Where/Which</t>
         </is>
       </c>
       <c r="C140" s="6" t="inlineStr">
         <is>
-          <t>"언제?", "몇 시?", "얼마 동안?"</t>
+          <t>"어디입니까?", "어느 나라?"</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>`qf_who`</t>
+          <t>`qf_central_thought`</t>
         </is>
       </c>
       <c r="B141" s="6" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Central Thought</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
-          <t>"누구입니까?"</t>
+          <t>"중심 생각으로 맞는 것"</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>`qf_how_many`</t>
+          <t>`qf_why`</t>
         </is>
       </c>
       <c r="B142" s="6" t="inlineStr">
         <is>
-          <t>How Many</t>
+          <t>Why/Reason</t>
         </is>
       </c>
       <c r="C142" s="6" t="inlineStr">
         <is>
-          <t>"몇 명?", "몇 개?"</t>
+          <t>"왜?", "이유"</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
+          <t>`qf_when_time`</t>
+        </is>
+      </c>
+      <c r="B143" s="6" t="inlineStr">
+        <is>
+          <t>When/Time</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="inlineStr">
+        <is>
+          <t>"언제?", "몇 시?", "얼마 동안?"</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="6" t="inlineStr">
+        <is>
+          <t>`qf_who`</t>
+        </is>
+      </c>
+      <c r="B144" s="6" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="C144" s="6" t="inlineStr">
+        <is>
+          <t>"누구입니까?"</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="6" t="inlineStr">
+        <is>
+          <t>`qf_how_many`</t>
+        </is>
+      </c>
+      <c r="B145" s="6" t="inlineStr">
+        <is>
+          <t>How Many</t>
+        </is>
+      </c>
+      <c r="C145" s="6" t="inlineStr">
+        <is>
+          <t>"몇 명?", "몇 개?"</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="6" t="inlineStr">
+        <is>
           <t>`qf_how_much`</t>
         </is>
       </c>
-      <c r="B143" s="6" t="inlineStr">
+      <c r="B146" s="6" t="inlineStr">
         <is>
           <t>How Much (Price)</t>
         </is>
       </c>
-      <c r="C143" s="6" t="inlineStr">
+      <c r="C146" s="6" t="inlineStr">
         <is>
           <t>"얼마입니까?"</t>
         </is>
       </c>
     </row>
-    <row r="145" ht="22" customHeight="1">
-      <c r="A145" s="13" t="inlineStr">
+    <row r="148" ht="22" customHeight="1">
+      <c r="A148" s="13" t="inlineStr">
         <is>
           <t>Nhóm câu hỏi KHÔNG có q_text</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" s="14" t="inlineStr">
+    <row r="149">
+      <c r="A149" s="14" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B146" s="14" t="inlineStr">
+      <c r="B149" s="14" t="inlineStr">
         <is>
           <t>Kind áp dụng</t>
         </is>
       </c>
-      <c r="C146" s="14" t="inlineStr">
+      <c r="C149" s="14" t="inlineStr">
         <is>
           <t>Mô tả</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="6" t="inlineStr">
-        <is>
-          <t>`qf_direct_qa`</t>
-        </is>
-      </c>
-      <c r="B147" s="6" t="inlineStr">
-        <is>
-          <t>310004</t>
-        </is>
-      </c>
-      <c r="C147" s="6" t="inlineStr">
-        <is>
-          <t>Nghe câu hỏi -&gt; chọn câu trả lời trực tiếp</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="6" t="inlineStr">
-        <is>
-          <t>`qf_next_utterance`</t>
-        </is>
-      </c>
-      <c r="B148" s="6" t="inlineStr">
-        <is>
-          <t>3410005</t>
-        </is>
-      </c>
-      <c r="C148" s="6" t="inlineStr">
-        <is>
-          <t>Nghe hội thoại -&gt; chọn câu nối tiếp</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="6" t="inlineStr">
-        <is>
-          <t>`qf_match_image`</t>
-        </is>
-      </c>
-      <c r="B149" s="6" t="inlineStr">
-        <is>
-          <t>310003</t>
-        </is>
-      </c>
-      <c r="C149" s="6" t="inlineStr">
-        <is>
-          <t>Nghe -&gt; chọn hình khớp</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="6" t="inlineStr">
         <is>
-          <t>`qf_match_content`</t>
+          <t>`qf_direct_qa`</t>
         </is>
       </c>
       <c r="B150" s="6" t="inlineStr">
         <is>
-          <t>310005</t>
+          <t>310004</t>
         </is>
       </c>
       <c r="C150" s="6" t="inlineStr">
         <is>
-          <t>Nghe -&gt; chọn phát biểu khớp nội dung</t>
+          <t>Nghe câu hỏi -&gt; chọn câu trả lời trực tiếp</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="6" t="inlineStr">
         <is>
-          <t>`qf_identify_sound`</t>
+          <t>`qf_next_utterance`</t>
         </is>
       </c>
       <c r="B151" s="6" t="inlineStr">
         <is>
-          <t>310001</t>
+          <t>3410005</t>
         </is>
       </c>
       <c r="C151" s="6" t="inlineStr">
         <is>
-          <t>Nghe -&gt; nhận diện từ/câu</t>
+          <t>Nghe hội thoại -&gt; chọn câu nối tiếp</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="6" t="inlineStr">
         <is>
-          <t>`qf_identify_time`</t>
+          <t>`qf_match_image`</t>
         </is>
       </c>
       <c r="B152" s="6" t="inlineStr">
         <is>
-          <t>3410002</t>
+          <t>310003</t>
         </is>
       </c>
       <c r="C152" s="6" t="inlineStr">
         <is>
-          <t>Nghe giờ -&gt; chọn đồng hồ</t>
+          <t>Nghe -&gt; chọn hình khớp</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="6" t="inlineStr">
         <is>
-          <t>`qf_image_qa`</t>
+          <t>`qf_match_content`</t>
         </is>
       </c>
       <c r="B153" s="6" t="inlineStr">
         <is>
-          <t>310002</t>
+          <t>310005</t>
         </is>
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>Nhìn hình + nghe 4 câu mô tả -&gt; chọn đúng</t>
+          <t>Nghe -&gt; chọn phát biểu khớp nội dung</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="6" t="inlineStr">
         <is>
+          <t>`qf_identify_sound`</t>
+        </is>
+      </c>
+      <c r="B154" s="6" t="inlineStr">
+        <is>
+          <t>310001</t>
+        </is>
+      </c>
+      <c r="C154" s="6" t="inlineStr">
+        <is>
+          <t>Nghe -&gt; nhận diện từ/câu</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="6" t="inlineStr">
+        <is>
+          <t>`qf_identify_time`</t>
+        </is>
+      </c>
+      <c r="B155" s="6" t="inlineStr">
+        <is>
+          <t>3410002</t>
+        </is>
+      </c>
+      <c r="C155" s="6" t="inlineStr">
+        <is>
+          <t>Nghe giờ -&gt; chọn đồng hồ</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="6" t="inlineStr">
+        <is>
+          <t>`qf_image_qa`</t>
+        </is>
+      </c>
+      <c r="B156" s="6" t="inlineStr">
+        <is>
+          <t>310002</t>
+        </is>
+      </c>
+      <c r="C156" s="6" t="inlineStr">
+        <is>
+          <t>Nhìn hình + nghe 4 câu mô tả -&gt; chọn đúng</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="6" t="inlineStr">
+        <is>
           <t>`qf_multi_comprehension`</t>
         </is>
       </c>
-      <c r="B154" s="6" t="inlineStr">
+      <c r="B157" s="6" t="inlineStr">
         <is>
           <t>310006</t>
         </is>
       </c>
-      <c r="C154" s="6" t="inlineStr">
+      <c r="C157" s="6" t="inlineStr">
         <is>
           <t>Nghe dài và trả lời 2 câu hỏi</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="11" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="157" ht="22" customHeight="1">
-      <c r="A157" s="9" t="inlineStr">
-        <is>
-          <t>Cấu trúc ngữ pháp trong audio (grammar_semantic)</t>
-        </is>
-      </c>
-      <c r="B157" s="10" t="n"/>
-      <c r="C157" s="10" t="n"/>
-      <c r="D157" s="10" t="n"/>
-      <c r="E157" s="10" t="n"/>
-      <c r="F157" s="10" t="n"/>
-    </row>
-    <row r="158" ht="22" customHeight="1">
-      <c r="A158" s="13" t="inlineStr">
-        <is>
-          <t>Phân bố Level 3 (2.242 câu, chỉ liệt kê &gt;=5%)</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="11" t="inlineStr">
         <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="22" customHeight="1">
+      <c r="A160" s="9" t="inlineStr">
+        <is>
+          <t>Cấu trúc ngữ pháp trong audio (grammar_semantic)</t>
+        </is>
+      </c>
+      <c r="B160" s="10" t="n"/>
+      <c r="C160" s="10" t="n"/>
+      <c r="D160" s="10" t="n"/>
+      <c r="E160" s="10" t="n"/>
+      <c r="F160" s="10" t="n"/>
+    </row>
+    <row r="161" ht="22" customHeight="1">
+      <c r="A161" s="13" t="inlineStr">
+        <is>
+          <t>Phân bố Level 3 (2.242 câu, chỉ liệt kê &gt;=5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="11" t="inlineStr">
+        <is>
           <t>gram_honorific_시(21%), gram_request_세요(19%), gram_honorific_습니다(18%), gram_cause_니까(8%), gram_cond_면(7%), gram_contrast_는데(7%), gram_prog_고있(6%), gram_intent_겠(6%), gram_cause_어서(5%)</t>
         </is>
       </c>
     </row>
-    <row r="160" ht="22" customHeight="1">
-      <c r="A160" s="13" t="inlineStr">
+    <row r="163" ht="22" customHeight="1">
+      <c r="A163" s="13" t="inlineStr">
         <is>
           <t>Bảng nhãn ngữ pháp theo ý nghĩa (Level 3)</t>
         </is>
       </c>
     </row>
-    <row r="161">
-      <c r="A161" s="14" t="inlineStr">
+    <row r="164">
+      <c r="A164" s="14" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B161" s="14" t="inlineStr">
+      <c r="B164" s="14" t="inlineStr">
         <is>
           <t>Cấu trúc</t>
         </is>
       </c>
-      <c r="C161" s="14" t="inlineStr">
+      <c r="C164" s="14" t="inlineStr">
         <is>
           <t>Ý nghĩa</t>
         </is>
       </c>
-      <c r="D161" s="14" t="inlineStr">
+      <c r="D164" s="14" t="inlineStr">
         <is>
           <t>L3</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="6" t="inlineStr">
-        <is>
-          <t>`gram_cause_어서`</t>
-        </is>
-      </c>
-      <c r="B162" s="6" t="inlineStr">
-        <is>
-          <t>~어서/아서</t>
-        </is>
-      </c>
-      <c r="C162" s="6" t="inlineStr">
-        <is>
-          <t>Nguyên nhân (nhẹ)</t>
-        </is>
-      </c>
-      <c r="D162" s="6" t="inlineStr">
-        <is>
-          <t>5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="6" t="inlineStr">
-        <is>
-          <t>`gram_cause_니까`</t>
-        </is>
-      </c>
-      <c r="B163" s="6" t="inlineStr">
-        <is>
-          <t>~니까</t>
-        </is>
-      </c>
-      <c r="C163" s="6" t="inlineStr">
-        <is>
-          <t>Nguyên nhân (nhấn mạnh)</t>
-        </is>
-      </c>
-      <c r="D163" s="6" t="inlineStr">
-        <is>
-          <t>8%</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="6" t="inlineStr">
-        <is>
-          <t>`gram_cond_면`</t>
-        </is>
-      </c>
-      <c r="B164" s="6" t="inlineStr">
-        <is>
-          <t>~(으)면</t>
-        </is>
-      </c>
-      <c r="C164" s="6" t="inlineStr">
-        <is>
-          <t>Điều kiện</t>
-        </is>
-      </c>
-      <c r="D164" s="6" t="inlineStr">
-        <is>
-          <t>7%</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="6" t="inlineStr">
         <is>
-          <t>`gram_contrast_지만`</t>
+          <t>`gram_cause_어서`</t>
         </is>
       </c>
       <c r="B165" s="6" t="inlineStr">
         <is>
-          <t>~지만</t>
+          <t>~어서/아서</t>
         </is>
       </c>
       <c r="C165" s="6" t="inlineStr">
         <is>
-          <t>Đối lập trực tiếp</t>
+          <t>Nguyên nhân (nhẹ)</t>
         </is>
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>5%</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="6" t="inlineStr">
         <is>
-          <t>`gram_contrast_는데`</t>
+          <t>`gram_cause_니까`</t>
         </is>
       </c>
       <c r="B166" s="6" t="inlineStr">
         <is>
-          <t>~는데/은데</t>
+          <t>~니까</t>
         </is>
       </c>
       <c r="C166" s="6" t="inlineStr">
         <is>
-          <t>Bối cảnh/đối lập mềm</t>
+          <t>Nguyên nhân (nhấn mạnh)</t>
         </is>
       </c>
       <c r="D166" s="6" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>8%</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="6" t="inlineStr">
         <is>
-          <t>`gram_intent_려고`</t>
+          <t>`gram_cond_면`</t>
         </is>
       </c>
       <c r="B167" s="6" t="inlineStr">
         <is>
-          <t>~(으)려고</t>
+          <t>~(으)면</t>
         </is>
       </c>
       <c r="C167" s="6" t="inlineStr">
         <is>
-          <t>Ý định</t>
+          <t>Điều kiện</t>
         </is>
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>7%</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="6" t="inlineStr">
         <is>
-          <t>`gram_intent_겠`</t>
+          <t>`gram_contrast_지만`</t>
         </is>
       </c>
       <c r="B168" s="6" t="inlineStr">
         <is>
-          <t>~겠어요/겠습니다</t>
+          <t>~지만</t>
         </is>
       </c>
       <c r="C168" s="6" t="inlineStr">
         <is>
-          <t>Dự định/suy đoán</t>
+          <t>Đối lập trực tiếp</t>
         </is>
       </c>
       <c r="D168" s="6" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>3%</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="6" t="inlineStr">
         <is>
-          <t>`gram_request_세요`</t>
+          <t>`gram_contrast_는데`</t>
         </is>
       </c>
       <c r="B169" s="6" t="inlineStr">
         <is>
-          <t>~(으)세요</t>
+          <t>~는데/은데</t>
         </is>
       </c>
       <c r="C169" s="6" t="inlineStr">
         <is>
-          <t>Yêu cầu lịch sự</t>
+          <t>Bối cảnh/đối lập mềm</t>
         </is>
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>7%</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="6" t="inlineStr">
         <is>
-          <t>`gram_request_주세요`</t>
+          <t>`gram_intent_려고`</t>
         </is>
       </c>
       <c r="B170" s="6" t="inlineStr">
         <is>
-          <t>~주세요</t>
+          <t>~(으)려고</t>
         </is>
       </c>
       <c r="C170" s="6" t="inlineStr">
         <is>
-          <t>Nhờ vả cụ thể</t>
+          <t>Ý định</t>
         </is>
       </c>
       <c r="D170" s="6" t="inlineStr">
@@ -3077,17 +3062,17 @@
     <row r="171">
       <c r="A171" s="6" t="inlineStr">
         <is>
-          <t>`gram_prog_고있`</t>
+          <t>`gram_intent_겠`</t>
         </is>
       </c>
       <c r="B171" s="6" t="inlineStr">
         <is>
-          <t>~고 있다</t>
+          <t>~겠어요/겠습니다</t>
         </is>
       </c>
       <c r="C171" s="6" t="inlineStr">
         <is>
-          <t>Đang diễn ra</t>
+          <t>Dự định/suy đoán</t>
         </is>
       </c>
       <c r="D171" s="6" t="inlineStr">
@@ -3099,891 +3084,940 @@
     <row r="172">
       <c r="A172" s="6" t="inlineStr">
         <is>
-          <t>`gram_honorific_시`</t>
+          <t>`gram_request_세요`</t>
         </is>
       </c>
       <c r="B172" s="6" t="inlineStr">
         <is>
-          <t>~시/셨/세요</t>
+          <t>~(으)세요</t>
         </is>
       </c>
       <c r="C172" s="6" t="inlineStr">
         <is>
-          <t>Kính ngữ (시)</t>
+          <t>Yêu cầu lịch sự</t>
         </is>
       </c>
       <c r="D172" s="6" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>19%</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="6" t="inlineStr">
         <is>
+          <t>`gram_request_주세요`</t>
+        </is>
+      </c>
+      <c r="B173" s="6" t="inlineStr">
+        <is>
+          <t>~주세요</t>
+        </is>
+      </c>
+      <c r="C173" s="6" t="inlineStr">
+        <is>
+          <t>Nhờ vả cụ thể</t>
+        </is>
+      </c>
+      <c r="D173" s="6" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="6" t="inlineStr">
+        <is>
+          <t>`gram_prog_고있`</t>
+        </is>
+      </c>
+      <c r="B174" s="6" t="inlineStr">
+        <is>
+          <t>~고 있다</t>
+        </is>
+      </c>
+      <c r="C174" s="6" t="inlineStr">
+        <is>
+          <t>Đang diễn ra</t>
+        </is>
+      </c>
+      <c r="D174" s="6" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="inlineStr">
+        <is>
+          <t>`gram_honorific_시`</t>
+        </is>
+      </c>
+      <c r="B175" s="6" t="inlineStr">
+        <is>
+          <t>~시/셨/세요</t>
+        </is>
+      </c>
+      <c r="C175" s="6" t="inlineStr">
+        <is>
+          <t>Kính ngữ (시)</t>
+        </is>
+      </c>
+      <c r="D175" s="6" t="inlineStr">
+        <is>
+          <t>21%</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="6" t="inlineStr">
+        <is>
           <t>`gram_honorific_습니다`</t>
         </is>
       </c>
-      <c r="B173" s="6" t="inlineStr">
+      <c r="B176" s="6" t="inlineStr">
         <is>
           <t>~습니다/ㅂ니다</t>
         </is>
       </c>
-      <c r="C173" s="6" t="inlineStr">
+      <c r="C176" s="6" t="inlineStr">
         <is>
           <t>Kính ngữ trang trọng</t>
         </is>
       </c>
-      <c r="D173" s="6" t="inlineStr">
+      <c r="D176" s="6" t="inlineStr">
         <is>
           <t>18%</t>
         </is>
       </c>
     </row>
-    <row r="175" ht="22" customHeight="1">
-      <c r="A175" s="13" t="inlineStr">
+    <row r="178" ht="22" customHeight="1">
+      <c r="A178" s="13" t="inlineStr">
         <is>
           <t>Ngữ pháp trong đáp án (answer_grammar)</t>
         </is>
       </c>
     </row>
-    <row r="176">
-      <c r="A176" s="14" t="inlineStr">
+    <row r="179">
+      <c r="A179" s="14" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B176" s="14" t="inlineStr">
+      <c r="B179" s="14" t="inlineStr">
         <is>
           <t>Mô tả</t>
         </is>
       </c>
-      <c r="C176" s="14" t="inlineStr">
+      <c r="C179" s="14" t="inlineStr">
         <is>
           <t>Kind áp dụng</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="6" t="inlineStr">
-        <is>
-          <t>`ans_word_phrase`</t>
-        </is>
-      </c>
-      <c r="B177" s="6" t="inlineStr">
-        <is>
-          <t>Đáp án là từ đơn / cụm ngắn</t>
-        </is>
-      </c>
-      <c r="C177" s="6" t="inlineStr">
-        <is>
-          <t>310001</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="6" t="inlineStr">
-        <is>
-          <t>`ans_formal_polite`</t>
-        </is>
-      </c>
-      <c r="B178" s="6" t="inlineStr">
-        <is>
-          <t>Đáp án dùng ~ㅂ니다/습니다</t>
-        </is>
-      </c>
-      <c r="C178" s="6" t="inlineStr">
-        <is>
-          <t>310002</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="6" t="inlineStr">
-        <is>
-          <t>`ans_image`</t>
-        </is>
-      </c>
-      <c r="B179" s="6" t="inlineStr">
-        <is>
-          <t>Đáp án là hình ảnh</t>
-        </is>
-      </c>
-      <c r="C179" s="6" t="inlineStr">
-        <is>
-          <t>310003, 3410002</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="6" t="inlineStr">
         <is>
-          <t>`ans_formal`</t>
+          <t>`ans_word_phrase`</t>
         </is>
       </c>
       <c r="B180" s="6" t="inlineStr">
         <is>
-          <t>Đáp án dùng ~ㅂ니다</t>
+          <t>Đáp án là từ đơn / cụm ngắn</t>
         </is>
       </c>
       <c r="C180" s="6" t="inlineStr">
         <is>
-          <t>310004, 310005, 310006</t>
+          <t>310001</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="6" t="inlineStr">
         <is>
+          <t>`ans_formal_polite`</t>
+        </is>
+      </c>
+      <c r="B181" s="6" t="inlineStr">
+        <is>
+          <t>Đáp án dùng ~ㅂ니다/습니다</t>
+        </is>
+      </c>
+      <c r="C181" s="6" t="inlineStr">
+        <is>
+          <t>310002</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="6" t="inlineStr">
+        <is>
+          <t>`ans_image`</t>
+        </is>
+      </c>
+      <c r="B182" s="6" t="inlineStr">
+        <is>
+          <t>Đáp án là hình ảnh</t>
+        </is>
+      </c>
+      <c r="C182" s="6" t="inlineStr">
+        <is>
+          <t>310003, 3410002</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="6" t="inlineStr">
+        <is>
+          <t>`ans_formal`</t>
+        </is>
+      </c>
+      <c r="B183" s="6" t="inlineStr">
+        <is>
+          <t>Đáp án dùng ~ㅂ니다</t>
+        </is>
+      </c>
+      <c r="C183" s="6" t="inlineStr">
+        <is>
+          <t>310004, 310005, 310006</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="6" t="inlineStr">
+        <is>
           <t>`ans_informal_polite`</t>
         </is>
       </c>
-      <c r="B181" s="6" t="inlineStr">
+      <c r="B184" s="6" t="inlineStr">
         <is>
           <t>Đáp án dùng ~아/어요</t>
         </is>
       </c>
-      <c r="C181" s="6" t="inlineStr">
+      <c r="C184" s="6" t="inlineStr">
         <is>
           <t>3410005</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="A183" s="11" t="inlineStr">
+    <row r="186">
+      <c r="A186" s="11" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="184" ht="22" customHeight="1">
-      <c r="A184" s="9" t="inlineStr">
+    <row r="187" ht="22" customHeight="1">
+      <c r="A187" s="9" t="inlineStr">
         <is>
           <t>Cấu trúc audio (audio_format)</t>
         </is>
       </c>
-      <c r="B184" s="10" t="n"/>
-      <c r="C184" s="10" t="n"/>
-      <c r="D184" s="10" t="n"/>
-      <c r="E184" s="10" t="n"/>
-      <c r="F184" s="10" t="n"/>
-    </row>
-    <row r="185">
-      <c r="A185" s="14" t="inlineStr">
+      <c r="B187" s="10" t="n"/>
+      <c r="C187" s="10" t="n"/>
+      <c r="D187" s="10" t="n"/>
+      <c r="E187" s="10" t="n"/>
+      <c r="F187" s="10" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="14" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B185" s="14" t="inlineStr">
+      <c r="B188" s="14" t="inlineStr">
         <is>
           <t>Mô tả</t>
         </is>
       </c>
-      <c r="C185" s="14" t="inlineStr">
+      <c r="C188" s="14" t="inlineStr">
         <is>
           <t>Kind chính</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="6" t="inlineStr">
-        <is>
-          <t>`audio_dialog_가나`</t>
-        </is>
-      </c>
-      <c r="B186" s="6" t="inlineStr">
-        <is>
-          <t>Hội thoại 가/나 (EPS)</t>
-        </is>
-      </c>
-      <c r="C186" s="6" t="inlineStr">
-        <is>
-          <t>310003-310006</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="6" t="inlineStr">
-        <is>
-          <t>`audio_single_word`</t>
-        </is>
-      </c>
-      <c r="B187" s="6" t="inlineStr">
-        <is>
-          <t>Từ đơn/cụm ngắn (&lt;15 ký tự)</t>
-        </is>
-      </c>
-      <c r="C187" s="6" t="inlineStr">
-        <is>
-          <t>310001, 3410002</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="6" t="inlineStr">
-        <is>
-          <t>`audio_single_sentence`</t>
-        </is>
-      </c>
-      <c r="B188" s="6" t="inlineStr">
-        <is>
-          <t>Câu đơn (15-50 ký tự)</t>
-        </is>
-      </c>
-      <c r="C188" s="6" t="inlineStr">
-        <is>
-          <t>310004, 3410005</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="6" t="inlineStr">
         <is>
+          <t>`audio_dialog_가나`</t>
+        </is>
+      </c>
+      <c r="B189" s="6" t="inlineStr">
+        <is>
+          <t>Hội thoại 가/나 (EPS)</t>
+        </is>
+      </c>
+      <c r="C189" s="6" t="inlineStr">
+        <is>
+          <t>310003-310006</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="6" t="inlineStr">
+        <is>
+          <t>`audio_single_word`</t>
+        </is>
+      </c>
+      <c r="B190" s="6" t="inlineStr">
+        <is>
+          <t>Từ đơn/cụm ngắn (&lt;15 ký tự)</t>
+        </is>
+      </c>
+      <c r="C190" s="6" t="inlineStr">
+        <is>
+          <t>310001, 3410002</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="6" t="inlineStr">
+        <is>
+          <t>`audio_single_sentence`</t>
+        </is>
+      </c>
+      <c r="B191" s="6" t="inlineStr">
+        <is>
+          <t>Câu đơn (15-50 ký tự)</t>
+        </is>
+      </c>
+      <c r="C191" s="6" t="inlineStr">
+        <is>
+          <t>310004, 3410005</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="6" t="inlineStr">
+        <is>
           <t>`audio_numbered`</t>
         </is>
       </c>
-      <c r="B189" s="6" t="inlineStr">
+      <c r="B192" s="6" t="inlineStr">
         <is>
           <t>4 câu mô tả đánh số (1. 2. 3. 4.)</t>
         </is>
       </c>
-      <c r="C189" s="6" t="inlineStr">
+      <c r="C192" s="6" t="inlineStr">
         <is>
           <t>310002</t>
         </is>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="11" t="inlineStr">
+    <row r="194">
+      <c r="A194" s="11" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="192" ht="22" customHeight="1">
-      <c r="A192" s="9" t="inlineStr">
+    <row r="195" ht="22" customHeight="1">
+      <c r="A195" s="9" t="inlineStr">
         <is>
           <t>Thang đo khó (Difficulty Scale) — EPS kinds only</t>
         </is>
       </c>
-      <c r="B192" s="10" t="n"/>
-      <c r="C192" s="10" t="n"/>
-      <c r="D192" s="10" t="n"/>
-      <c r="E192" s="10" t="n"/>
-      <c r="F192" s="10" t="n"/>
-    </row>
-    <row r="193">
-      <c r="A193" s="14" t="inlineStr">
+      <c r="B195" s="10" t="n"/>
+      <c r="C195" s="10" t="n"/>
+      <c r="D195" s="10" t="n"/>
+      <c r="E195" s="10" t="n"/>
+      <c r="F195" s="10" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="14" t="inlineStr">
         <is>
           <t>Mức</t>
         </is>
       </c>
-      <c r="B193" s="14" t="inlineStr">
+      <c r="B196" s="14" t="inlineStr">
         <is>
           <t>Kind</t>
         </is>
       </c>
-      <c r="C193" s="14" t="inlineStr">
+      <c r="C196" s="14" t="inlineStr">
         <is>
           <t>Kiểu suy luận</t>
         </is>
       </c>
-      <c r="D193" s="14" t="inlineStr">
+      <c r="D196" s="14" t="inlineStr">
         <is>
           <t>Nhãn</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B194" s="6" t="inlineStr">
-        <is>
-          <t>310001, 3410002</t>
-        </is>
-      </c>
-      <c r="C194" s="6" t="inlineStr">
-        <is>
-          <t>`sound_recognition` / `time_recognition`</t>
-        </is>
-      </c>
-      <c r="D194" s="6" t="inlineStr">
-        <is>
-          <t>Nhận diện từ/giờ</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B195" s="6" t="inlineStr">
-        <is>
-          <t>310004, 310002</t>
-        </is>
-      </c>
-      <c r="C195" s="6" t="inlineStr">
-        <is>
-          <t>`direct_match` / `image_qa`</t>
-        </is>
-      </c>
-      <c r="D195" s="6" t="inlineStr">
-        <is>
-          <t>Hỏi-đáp đơn giản</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B196" s="6" t="inlineStr">
-        <is>
-          <t>3410005</t>
-        </is>
-      </c>
-      <c r="C196" s="6" t="inlineStr">
-        <is>
-          <t>`pragmatic_response`</t>
-        </is>
-      </c>
-      <c r="D196" s="6" t="inlineStr">
-        <is>
-          <t>Chọn câu nối tiếp</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B197" s="6" t="inlineStr">
         <is>
-          <t>310003</t>
+          <t>310001, 3410002</t>
         </is>
       </c>
       <c r="C197" s="6" t="inlineStr">
         <is>
-          <t>`scene_matching`</t>
+          <t>`sound_recognition` / `time_recognition`</t>
         </is>
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>Chọn hình liên quan</t>
+          <t>Nhận diện từ/giờ</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B198" s="6" t="inlineStr">
         <is>
-          <t>310005</t>
+          <t>310004, 310002</t>
         </is>
       </c>
       <c r="C198" s="6" t="inlineStr">
         <is>
-          <t>`detail_extraction`</t>
+          <t>`direct_match` / `image_qa`</t>
         </is>
       </c>
       <c r="D198" s="6" t="inlineStr">
         <is>
-          <t>Trích xuất chi tiết</t>
+          <t>Hỏi-đáp đơn giản</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="6" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B199" s="6" t="inlineStr">
+        <is>
+          <t>3410005</t>
+        </is>
+      </c>
+      <c r="C199" s="6" t="inlineStr">
+        <is>
+          <t>`pragmatic_response`</t>
+        </is>
+      </c>
+      <c r="D199" s="6" t="inlineStr">
+        <is>
+          <t>Chọn câu nối tiếp</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B200" s="6" t="inlineStr">
+        <is>
+          <t>310003</t>
+        </is>
+      </c>
+      <c r="C200" s="6" t="inlineStr">
+        <is>
+          <t>`scene_matching`</t>
+        </is>
+      </c>
+      <c r="D200" s="6" t="inlineStr">
+        <is>
+          <t>Chọn hình liên quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B201" s="6" t="inlineStr">
+        <is>
+          <t>310005</t>
+        </is>
+      </c>
+      <c r="C201" s="6" t="inlineStr">
+        <is>
+          <t>`detail_extraction`</t>
+        </is>
+      </c>
+      <c r="D201" s="6" t="inlineStr">
+        <is>
+          <t>Trích xuất chi tiết</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="6" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B199" s="6" t="inlineStr">
+      <c r="B202" s="6" t="inlineStr">
         <is>
           <t>310006</t>
         </is>
       </c>
-      <c r="C199" s="6" t="inlineStr">
+      <c r="C202" s="6" t="inlineStr">
         <is>
           <t>`multi_comprehension`</t>
         </is>
       </c>
-      <c r="D199" s="6" t="inlineStr">
+      <c r="D202" s="6" t="inlineStr">
         <is>
           <t>2 câu hỏi / đoạn dài</t>
         </is>
       </c>
     </row>
-    <row r="201" ht="22" customHeight="1">
-      <c r="A201" s="13" t="inlineStr">
+    <row r="204" ht="22" customHeight="1">
+      <c r="A204" s="13" t="inlineStr">
         <is>
           <t>Mô tả kiểu suy luận (reasoning_type)</t>
         </is>
       </c>
     </row>
-    <row r="202">
-      <c r="A202" s="14" t="inlineStr">
+    <row r="205">
+      <c r="A205" s="14" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B202" s="14" t="inlineStr">
+      <c r="B205" s="14" t="inlineStr">
         <is>
           <t>Mô tả</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" s="6" t="inlineStr">
-        <is>
-          <t>`sound_recognition`</t>
-        </is>
-      </c>
-      <c r="B203" s="6" t="inlineStr">
-        <is>
-          <t>Nhận diện chính xác từ/câu được nghe</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="6" t="inlineStr">
-        <is>
-          <t>`time_recognition`</t>
-        </is>
-      </c>
-      <c r="B204" s="6" t="inlineStr">
-        <is>
-          <t>Nghe giờ, chọn đồng hồ phù hợp</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" s="6" t="inlineStr">
-        <is>
-          <t>`direct_match`</t>
-        </is>
-      </c>
-      <c r="B205" s="6" t="inlineStr">
-        <is>
-          <t>Ghép câu hỏi với câu trả lời trực tiếp</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="6" t="inlineStr">
         <is>
-          <t>`image_qa`</t>
+          <t>`sound_recognition`</t>
         </is>
       </c>
       <c r="B206" s="6" t="inlineStr">
         <is>
-          <t>Nhìn hình, nghe câu hỏi + đáp án, chọn đúng</t>
+          <t>Nhận diện chính xác từ/câu được nghe</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="6" t="inlineStr">
         <is>
-          <t>`pragmatic_response`</t>
+          <t>`time_recognition`</t>
         </is>
       </c>
       <c r="B207" s="6" t="inlineStr">
         <is>
-          <t>Chọn phản hồi phù hợp ngữ cảnh giao tiếp</t>
+          <t>Nghe giờ, chọn đồng hồ phù hợp</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="6" t="inlineStr">
         <is>
-          <t>`scene_matching`</t>
+          <t>`direct_match`</t>
         </is>
       </c>
       <c r="B208" s="6" t="inlineStr">
         <is>
-          <t>Nghe audio, chọn bức tranh minh họa khớp</t>
+          <t>Ghép câu hỏi với câu trả lời trực tiếp</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="6" t="inlineStr">
         <is>
-          <t>`detail_extraction`</t>
+          <t>`image_qa`</t>
         </is>
       </c>
       <c r="B209" s="6" t="inlineStr">
         <is>
-          <t>Trích xuất chi tiết cụ thể từ hội thoại</t>
+          <t>Nhìn hình, nghe câu hỏi + đáp án, chọn đúng</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="6" t="inlineStr">
         <is>
+          <t>`pragmatic_response`</t>
+        </is>
+      </c>
+      <c r="B210" s="6" t="inlineStr">
+        <is>
+          <t>Chọn phản hồi phù hợp ngữ cảnh giao tiếp</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="6" t="inlineStr">
+        <is>
+          <t>`scene_matching`</t>
+        </is>
+      </c>
+      <c r="B211" s="6" t="inlineStr">
+        <is>
+          <t>Nghe audio, chọn bức tranh minh họa khớp</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="6" t="inlineStr">
+        <is>
+          <t>`detail_extraction`</t>
+        </is>
+      </c>
+      <c r="B212" s="6" t="inlineStr">
+        <is>
+          <t>Trích xuất chi tiết cụ thể từ hội thoại</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="6" t="inlineStr">
+        <is>
           <t>`multi_comprehension`</t>
         </is>
       </c>
-      <c r="B210" s="6" t="inlineStr">
+      <c r="B213" s="6" t="inlineStr">
         <is>
           <t>Trả lời 2 câu hỏi từ 1 đoạn</t>
         </is>
       </c>
     </row>
-    <row r="212">
-      <c r="A212" s="11" t="inlineStr">
+    <row r="215">
+      <c r="A215" s="11" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="213" ht="22" customHeight="1">
-      <c r="A213" s="9" t="inlineStr">
+    <row r="216" ht="22" customHeight="1">
+      <c r="A216" s="9" t="inlineStr">
         <is>
           <t>Cấp độ giao tiếp trong audio (speech_level)</t>
         </is>
       </c>
-      <c r="B213" s="10" t="n"/>
-      <c r="C213" s="10" t="n"/>
-      <c r="D213" s="10" t="n"/>
-      <c r="E213" s="10" t="n"/>
-      <c r="F213" s="10" t="n"/>
-    </row>
-    <row r="214">
-      <c r="A214" s="14" t="inlineStr">
+      <c r="B216" s="10" t="n"/>
+      <c r="C216" s="10" t="n"/>
+      <c r="D216" s="10" t="n"/>
+      <c r="E216" s="10" t="n"/>
+      <c r="F216" s="10" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="14" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="B214" s="14" t="inlineStr">
+      <c r="B217" s="14" t="inlineStr">
         <is>
           <t>Audio chính</t>
         </is>
       </c>
-      <c r="C214" s="14" t="inlineStr">
+      <c r="C217" s="14" t="inlineStr">
         <is>
           <t>Đáp án</t>
         </is>
       </c>
     </row>
-    <row r="215">
-      <c r="A215" s="6" t="inlineStr">
+    <row r="218">
+      <c r="A218" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B215" s="6" t="inlineStr">
+      <c r="B218" s="6" t="inlineStr">
         <is>
           <t>`informal_polite` 37%, `modifier` 31%, `connective` 16%</t>
         </is>
       </c>
-      <c r="C215" s="6" t="inlineStr">
+      <c r="C218" s="6" t="inlineStr">
         <is>
           <t>`formal_polite` (~ㅂ니다) cho EPS</t>
         </is>
       </c>
     </row>
-    <row r="217">
-      <c r="A217" s="11" t="inlineStr">
+    <row r="220">
+      <c r="A220" s="11" t="inlineStr">
         <is>
           <t>Quy tắc: Audio EPS dùng informal_polite là chính. Đáp án EPS thường dùng formal_polite (~ㅂ니다) — xem answer_grammar ans_formal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" s="11" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="219" ht="22" customHeight="1">
-      <c r="A219" s="9" t="inlineStr">
-        <is>
-          <t>Quy tắc chung khi gen câu hỏi</t>
-        </is>
-      </c>
-      <c r="B219" s="10" t="n"/>
-      <c r="C219" s="10" t="n"/>
-      <c r="D219" s="10" t="n"/>
-      <c r="E219" s="10" t="n"/>
-      <c r="F219" s="10" t="n"/>
-    </row>
-    <row r="220" ht="22" customHeight="1">
-      <c r="A220" s="13" t="inlineStr">
-        <is>
-          <t>1. Chất lượng nội dung tiếng Hàn</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="11" t="inlineStr">
         <is>
-          <t>• Dùng ngữ pháp đúng Level 3 (xem bảng speech_level + grammar_semantic)</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" s="11" t="inlineStr">
-        <is>
-          <t>• Hội thoại tự nhiên, đa dạng chủ đề đời sống + lao động</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" s="11" t="inlineStr">
-        <is>
-          <t>• KHÔNG lặp lại từ vựng/ngữ cảnh giữa các câu trong cùng batch</t>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="22" customHeight="1">
+      <c r="A222" s="9" t="inlineStr">
+        <is>
+          <t>Quy tắc chung khi gen câu hỏi</t>
+        </is>
+      </c>
+      <c r="B222" s="10" t="n"/>
+      <c r="C222" s="10" t="n"/>
+      <c r="D222" s="10" t="n"/>
+      <c r="E222" s="10" t="n"/>
+      <c r="F222" s="10" t="n"/>
+    </row>
+    <row r="223" ht="22" customHeight="1">
+      <c r="A223" s="13" t="inlineStr">
+        <is>
+          <t>1. Chất lượng nội dung tiếng Hàn</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="11" t="inlineStr">
         <is>
-          <t>• Pha trộn chủ đề chung + chủ đề EPS đặc thù</t>
-        </is>
-      </c>
-    </row>
-    <row r="225" ht="22" customHeight="1">
-      <c r="A225" s="13" t="inlineStr">
-        <is>
-          <t>2. Xây dựng đáp án sai (distractor)</t>
+          <t>• Dùng ngữ pháp đúng Level 3 (xem bảng speech_level + grammar_semantic)</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="11" t="inlineStr">
+        <is>
+          <t>• Hội thoại tự nhiên, đa dạng chủ đề đời sống + lao động</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="11" t="inlineStr">
         <is>
-          <t>• Tuân theo tỷ lệ bẫy của từng kind (xem file kind tương ứng)</t>
+          <t>• KHÔNG lặp lại từ vựng/ngữ cảnh giữa các câu trong cùng batch</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="11" t="inlineStr">
         <is>
-          <t>• Phải hợp lý nhưng SAI về nội dung</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" s="11" t="inlineStr">
-        <is>
-          <t>• Tái sử dụng từ vựng audio khi kind yêu cầu shared_word</t>
-        </is>
-      </c>
-    </row>
-    <row r="229" ht="22" customHeight="1">
-      <c r="A229" s="13" t="inlineStr">
-        <is>
-          <t>3. Giải thích (explain)</t>
+          <t>• Pha trộn chủ đề chung + chủ đề EPS đặc thù</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="22" customHeight="1">
+      <c r="A228" s="13" t="inlineStr">
+        <is>
+          <t>2. Xây dựng đáp án sai (distractor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="11" t="inlineStr">
+        <is>
+          <t>• Tuân theo tỷ lệ bẫy của từng kind (xem file kind tương ứng)</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="11" t="inlineStr">
         <is>
-          <t>• vi: Dịch cả 4 đáp án -&gt; dấu -------------------- -&gt; giải thích đáp án đúng, ghi chú trap type cho từng đáp án sai</t>
+          <t>• Phải hợp lý nhưng SAI về nội dung</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="11" t="inlineStr">
         <is>
-          <t>• en: Tương tự bằng tiếng Anh</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" s="11" t="inlineStr">
-        <is>
-          <t>• Highlight từ vựng/ngữ pháp quan trọng</t>
-        </is>
-      </c>
-    </row>
-    <row r="233" ht="22" customHeight="1">
-      <c r="A233" s="13" t="inlineStr">
-        <is>
-          <t>4. Số lượng</t>
+          <t>• Tái sử dụng từ vựng audio khi kind yêu cầu shared_word</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="22" customHeight="1">
+      <c r="A232" s="13" t="inlineStr">
+        <is>
+          <t>3. Giải thích (explain)</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="11" t="inlineStr">
+        <is>
+          <t>• vi: Dịch cả 4 đáp án -&gt; dấu -------------------- -&gt; giải thích đáp án đúng, ghi chú trap type cho từng đáp án sai</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="11" t="inlineStr">
         <is>
-          <t>• Mặc định: 5 câu mỗi kind nếu user không chỉ định</t>
+          <t>• en: Tương tự bằng tiếng Anh</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="11" t="inlineStr">
         <is>
-          <t>• Tối đa: 20 câu mỗi lần</t>
+          <t>• Highlight từ vựng/ngữ pháp quan trọng</t>
         </is>
       </c>
     </row>
     <row r="236" ht="22" customHeight="1">
       <c r="A236" s="13" t="inlineStr">
         <is>
-          <t>5. Kiểm tra sau khi gen (Validation Checklist)</t>
+          <t>4. Số lượng</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="11" t="inlineStr">
         <is>
-          <t>• [ ] q_correct nằm trong 1-4</t>
+          <t>• Mặc định: 5 câu mỗi kind nếu user không chỉ định</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="11" t="inlineStr">
         <is>
-          <t>• [ ] 4 đáp án không trùng nhau</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" s="11" t="inlineStr">
-        <is>
-          <t>• [ ] Audio là tiếng Hàn tự nhiên</t>
+          <t>• Tối đa: 20 câu mỗi lần</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="22" customHeight="1">
+      <c r="A239" s="13" t="inlineStr">
+        <is>
+          <t>5. Kiểm tra sau khi gen (Validation Checklist)</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="11" t="inlineStr">
         <is>
-          <t>• [ ] Ngữ pháp đúng Level 3</t>
+          <t>• [ ] q_correct nằm trong 1-4</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="11" t="inlineStr">
         <is>
-          <t>• [ ] Bẫy đúng phân bố của kind</t>
+          <t>• [ ] 4 đáp án không trùng nhau</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="11" t="inlineStr">
         <is>
-          <t>• [ ] Bản dịch (vi/en) chính xác</t>
+          <t>• [ ] Audio là tiếng Hàn tự nhiên</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="11" t="inlineStr">
         <is>
-          <t>• [ ] explain chứa dịch 4 đáp án + lý do đáp án đúng + trap type cho đáp án sai</t>
+          <t>• [ ] Ngữ pháp đúng Level 3</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="11" t="inlineStr">
         <is>
-          <t>• [ ] count_question khớp số phần tử trong content</t>
+          <t>• [ ] Bẫy đúng phân bố của kind</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="11" t="inlineStr">
         <is>
-          <t>• [ ] level luôn = 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="246" ht="22" customHeight="1">
-      <c r="A246" s="9" t="inlineStr">
-        <is>
-          <t>Workflow</t>
-        </is>
-      </c>
-      <c r="B246" s="10" t="n"/>
-      <c r="C246" s="10" t="n"/>
-      <c r="D246" s="10" t="n"/>
-      <c r="E246" s="10" t="n"/>
-      <c r="F246" s="10" t="n"/>
+          <t>• [ ] Bản dịch (vi/en) chính xác</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="11" t="inlineStr">
+        <is>
+          <t>• [ ] explain chứa dịch 4 đáp án + lý do đáp án đúng + trap type cho đáp án sai</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="11" t="inlineStr">
         <is>
-          <t>1. User chỉ định kind -&gt; đọc file kinds/{kind}.md</t>
+          <t>• [ ] count_question khớp số phần tử trong content</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="11" t="inlineStr">
         <is>
-          <t>2. Hỏi số lượng (mặc định 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" s="11" t="inlineStr">
-        <is>
-          <t>3. Gen câu hỏi theo JSON format + quy tắc kind + chiến lược bẫy</t>
-        </is>
-      </c>
+          <t>• [ ] level luôn = 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="22" customHeight="1">
+      <c r="A249" s="9" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="B249" s="10" t="n"/>
+      <c r="C249" s="10" t="n"/>
+      <c r="D249" s="10" t="n"/>
+      <c r="E249" s="10" t="n"/>
+      <c r="F249" s="10" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="11" t="inlineStr">
         <is>
-          <t>4. Lưu JSON tạm -&gt; chạy scripts/save_listen.py để tách CSV theo kind</t>
+          <t>1. User chỉ định kind -&gt; đọc file kinds/{kind}.md</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="11" t="inlineStr">
         <is>
+          <t>2. Hỏi số lượng (mặc định 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="11" t="inlineStr">
+        <is>
+          <t>3. Gen câu hỏi theo JSON format + quy tắc kind + chiến lược bẫy</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="11" t="inlineStr">
+        <is>
+          <t>4. Lưu JSON tạm -&gt; chạy scripts/save_listen.py để tách CSV theo kind</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="11" t="inlineStr">
+        <is>
           <t>5. Validate theo checklist</t>
         </is>
       </c>
     </row>
-    <row r="252" ht="22" customHeight="1">
-      <c r="A252" s="13" t="inlineStr">
+    <row r="255" ht="22" customHeight="1">
+      <c r="A255" s="13" t="inlineStr">
         <is>
           <t>Lưu kết quả bằng script</t>
         </is>
       </c>
-    </row>
-    <row r="253">
-      <c r="A253" s="12" t="inlineStr">
-        <is>
-          <t># Lưu CSV theo kind + JSON + merge tổng</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" s="12" t="inlineStr">
-        <is>
-          <t>python skills/topik-listen-gen-eps/scripts/save_listen.py gen_temp.json -o output/listen-eps --json --merge</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" s="12" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" s="12" t="inlineStr">
         <is>
-          <t># Chỉ validate</t>
+          <t># Lưu CSV theo kind + JSON + merge tổng</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="12" t="inlineStr">
         <is>
-          <t>python skills/topik-listen-gen-eps/scripts/save_listen.py gen_temp.json --validate-only</t>
+          <t>python skills/topik-listen-gen-eps/scripts/save_listen.py gen_temp.json -o output/listen-eps --json --merge</t>
         </is>
       </c>
     </row>
@@ -3993,19 +4027,36 @@
     <row r="259">
       <c r="A259" s="12" t="inlineStr">
         <is>
-          <t># Append thêm batch mới</t>
+          <t># Chỉ validate</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="12" t="inlineStr">
         <is>
+          <t>python skills/topik-listen-gen-eps/scripts/save_listen.py gen_temp.json --validate-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="12" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="12" t="inlineStr">
+        <is>
+          <t># Append thêm batch mới</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="12" t="inlineStr">
+        <is>
           <t>python skills/topik-listen-gen-eps/scripts/save_listen.py new_batch.json --append</t>
         </is>
       </c>
     </row>
-    <row r="262">
-      <c r="A262" s="11" t="inlineStr">
+    <row r="265">
+      <c r="A265" s="11" t="inlineStr">
         <is>
           <t>Output: output/listen-eps/level_3/{kind}.csv</t>
         </is>
@@ -4013,12 +4064,11 @@
     </row>
   </sheetData>
   <mergeCells count="158">
-    <mergeCell ref="A183:F183"/>
     <mergeCell ref="A84:F84"/>
     <mergeCell ref="A66:F66"/>
     <mergeCell ref="A118:F118"/>
     <mergeCell ref="A75:F75"/>
-    <mergeCell ref="A158:F158"/>
+    <mergeCell ref="A133:F133"/>
     <mergeCell ref="A238:F238"/>
     <mergeCell ref="A50:F50"/>
     <mergeCell ref="A3:F3"/>
@@ -4027,15 +4077,18 @@
     <mergeCell ref="A239:F239"/>
     <mergeCell ref="A47:F47"/>
     <mergeCell ref="A160:F160"/>
-    <mergeCell ref="A175:F175"/>
     <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A263:F263"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="A159:F159"/>
     <mergeCell ref="A224:F224"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A134:F134"/>
     <mergeCell ref="A81:F81"/>
     <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A265:F265"/>
+    <mergeCell ref="A161:F161"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A249:F249"/>
@@ -4045,6 +4098,7 @@
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="A64:F64"/>
+    <mergeCell ref="A186:F186"/>
     <mergeCell ref="A257:F257"/>
     <mergeCell ref="A73:F73"/>
     <mergeCell ref="A226:F226"/>
@@ -4059,48 +4113,48 @@
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A212:F212"/>
     <mergeCell ref="A243:F243"/>
+    <mergeCell ref="A252:F252"/>
     <mergeCell ref="A221:F221"/>
-    <mergeCell ref="A252:F252"/>
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="A236:F236"/>
     <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A163:F163"/>
     <mergeCell ref="A223:F223"/>
+    <mergeCell ref="A195:F195"/>
     <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A204:F204"/>
     <mergeCell ref="A85:F85"/>
     <mergeCell ref="A42:F42"/>
-    <mergeCell ref="A213:F213"/>
-    <mergeCell ref="A126:F126"/>
+    <mergeCell ref="A259:F259"/>
     <mergeCell ref="A254:F254"/>
-    <mergeCell ref="A259:F259"/>
     <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A135:F135"/>
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A262:F262"/>
     <mergeCell ref="A62:F62"/>
     <mergeCell ref="A240:F240"/>
+    <mergeCell ref="A215:F215"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A230:F230"/>
     <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A127:F127"/>
     <mergeCell ref="A48:F48"/>
     <mergeCell ref="A30:F30"/>
     <mergeCell ref="A232:F232"/>
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A191:F191"/>
+    <mergeCell ref="A216:F216"/>
     <mergeCell ref="A225:F225"/>
+    <mergeCell ref="A178:F178"/>
     <mergeCell ref="A79:F79"/>
     <mergeCell ref="A61:F61"/>
     <mergeCell ref="A88:F88"/>
-    <mergeCell ref="A218:F218"/>
+    <mergeCell ref="A162:F162"/>
     <mergeCell ref="A227:F227"/>
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A46:F46"/>
-    <mergeCell ref="A217:F217"/>
     <mergeCell ref="A74:F74"/>
     <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A145:F145"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A71:F71"/>
     <mergeCell ref="A129:F129"/>
@@ -4125,7 +4179,6 @@
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A245:F245"/>
     <mergeCell ref="A92:F92"/>
-    <mergeCell ref="A157:F157"/>
     <mergeCell ref="A39:F39"/>
     <mergeCell ref="A49:F49"/>
     <mergeCell ref="A36:F36"/>
@@ -4137,7 +4190,6 @@
     <mergeCell ref="A87:F87"/>
     <mergeCell ref="A65:F65"/>
     <mergeCell ref="A246:F246"/>
-    <mergeCell ref="A128:F128"/>
     <mergeCell ref="A255:F255"/>
     <mergeCell ref="A80:F80"/>
     <mergeCell ref="A37:F37"/>
@@ -4145,30 +4197,29 @@
     <mergeCell ref="A89:F89"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A192:F192"/>
     <mergeCell ref="A248:F248"/>
     <mergeCell ref="A57:F57"/>
     <mergeCell ref="A235:F235"/>
     <mergeCell ref="A247:F247"/>
     <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A219:F219"/>
     <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A194:F194"/>
     <mergeCell ref="A234:F234"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A91:F91"/>
-    <mergeCell ref="A184:F184"/>
     <mergeCell ref="A43:F43"/>
-    <mergeCell ref="A156:F156"/>
     <mergeCell ref="A52:F52"/>
     <mergeCell ref="A67:F67"/>
     <mergeCell ref="A220:F220"/>
     <mergeCell ref="A130:F130"/>
     <mergeCell ref="A77:F77"/>
-    <mergeCell ref="A201:F201"/>
+    <mergeCell ref="A148:F148"/>
+    <mergeCell ref="A261:F261"/>
     <mergeCell ref="A222:F222"/>
     <mergeCell ref="A132:F132"/>
     <mergeCell ref="A110:F110"/>
     <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A187:F187"/>
     <mergeCell ref="A69:F69"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>
@@ -4716,7 +4767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4970,315 +5021,343 @@
       <c r="F24" s="10" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>Không phát hiện bẫy rõ — đáp án nằm trong audio, không phải text options.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Bẫy</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Tỷ lệ</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>`trap_detail_distort`</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Mô tả đúng bối cảnh nhưng sai chi tiết hành động</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>`trap_shared_noun`</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Đáp án dùng lại từ vựng trong audio nhưng sai nội dung</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>`trap_neg_없안`</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Đáp án đảo nghĩa so với nội dung audio</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Cấu trúc audio</t>
         </is>
       </c>
-      <c r="B26" s="10" t="n"/>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
-      <c r="E26" s="10" t="n"/>
-      <c r="F26" s="10" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>• 4 câu mô tả được đọc to (đánh số 1-4), mô tả điều có thể đang xảy ra trong hình</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>• Format:</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  1. 식사를 하고 있습니다.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  2. 빨래를 하고 있습니다.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  3. 머리를 자르고 있습니다.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">  4. 김치를 만들고 있습니다.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="9" t="inlineStr">
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
         <is>
           <t>Cấu trúc đáp án</t>
         </is>
       </c>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="10" t="n"/>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>• q_answer: ["1. ", "2. ", "3. ", "4. "] (310002) hoặc ["1.", "2.", "3.", "4."] (3410003) — đáp án nằm trong audio</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>• q_text: có câu hỏi về hình (e.g., "사람들이 무엇을 하고 있습니까?")</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>• q_image: có (1 ảnh mỗi câu)</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>Phân loại q_text (8 dạng)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="14" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>Dạng</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>Số câu</t>
         </is>
       </c>
-      <c r="C39" s="14" t="inlineStr">
+      <c r="C43" s="14" t="inlineStr">
         <is>
           <t>Ví dụ</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>`object_what`</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>94</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>이것은 무엇입니까?</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>`action_doing`</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>111</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>이 사람은 무엇을 하고 있습니까?</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>`place_where`</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="inlineStr">
-        <is>
-          <t>여기는 어디입니까?</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>`date_when`</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>언제입니까?</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>`object_job`</t>
+          <t>`object_what`</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>94</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>이 사람의 직업은 무엇입니까?</t>
+          <t>이것은 무엇입니까?</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>`weather`</t>
+          <t>`action_doing`</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>111</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>날씨가 어떻습니까?</t>
+          <t>이 사람은 무엇을 하고 있습니까?</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>`count`</t>
+          <t>`place_where`</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>100</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>몇 개입니까?</t>
+          <t>여기는 어디입니까?</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
+          <t>`date_when`</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>언제입니까?</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>`object_job`</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>이 사람의 직업은 무엇입니까?</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>`weather`</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>날씨가 어떻습니까?</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>`count`</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>몇 개입니까?</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
           <t>`quality`</t>
         </is>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>어떤 것입니까?</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="9" t="inlineStr">
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="9" t="inlineStr">
         <is>
           <t>Cách mô tả ảnh (q_image_description)</t>
         </is>
       </c>
-      <c r="B49" s="10" t="n"/>
-      <c r="C49" s="10" t="n"/>
-      <c r="D49" s="10" t="n"/>
-      <c r="E49" s="10" t="n"/>
-      <c r="F49" s="10" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="11" t="inlineStr">
-        <is>
-          <t>Mỗi câu có 1 bức tranh. Dùng key "image" để mô tả cảnh trong hình.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="9" t="inlineStr">
-        <is>
-          <t>Quy tắc tạo audio và hình</t>
-        </is>
-      </c>
-      <c r="B51" s="10" t="n"/>
-      <c r="C51" s="10" t="n"/>
-      <c r="D51" s="10" t="n"/>
-      <c r="E51" s="10" t="n"/>
-      <c r="F51" s="10" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="11" t="inlineStr">
-        <is>
-          <t>1. Hình phải mô tả cảnh rõ ràng, dễ nhận biết</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="11" t="inlineStr">
-        <is>
-          <t>2. Audio gồm 1 câu đúng + 3 câu hợp lý nhưng sai so với hình</t>
-        </is>
-      </c>
+      <c r="B53" s="10" t="n"/>
+      <c r="C53" s="10" t="n"/>
+      <c r="D53" s="10" t="n"/>
+      <c r="E53" s="10" t="n"/>
+      <c r="F53" s="10" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>3. 3 câu sai phải liên quan đến cùng chủ đề nhưng khác hành động/đối tượng/địa điểm</t>
+          <t>Mỗi câu có 1 bức tranh. Dùng key "image" để mô tả cảnh trong hình.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>Ví dụ</t>
+          <t>Quy tắc tạo audio và hình</t>
         </is>
       </c>
       <c r="B55" s="10" t="n"/>
@@ -5288,96 +5367,128 @@
       <c r="F55" s="10" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="inlineStr">
-        <is>
-          <t>{</t>
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>1. Hình phải mô tả cảnh rõ ràng, dễ nhận biết</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  "g_text_audio": "1. 식사를 하고 있습니다.\n2. 빨래를 하고 있습니다.\n3. 머리를 자르고 있습니다.\n4. 김치를 만들고 있습니다.",</t>
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>2. Audio gồm 1 câu đúng + 3 câu hợp lý nhưng sai so với hình</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  "content": [{</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    "q_text": "사람들이 무엇을 하고 있습니까?",</t>
-        </is>
-      </c>
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>3. 3 câu sai phải liên quan đến cùng chủ đề nhưng khác hành động/đối tượng/địa điểm</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>Ví dụ</t>
+        </is>
+      </c>
+      <c r="B59" s="10" t="n"/>
+      <c r="C59" s="10" t="n"/>
+      <c r="D59" s="10" t="n"/>
+      <c r="E59" s="10" t="n"/>
+      <c r="F59" s="10" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "q_image_description": {</t>
+          <t>{</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "image": "여자가 부엌에서 빨래를 하고 있다. 세탁기 옆에 빨래 바구니가 있다."</t>
+          <t xml:space="preserve">  "g_text_audio": "1. 식사를 하고 있습니다.\n2. 빨래를 하고 있습니다.\n3. 머리를 자르고 있습니다.\n4. 김치를 만들고 있습니다.",</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    },</t>
+          <t xml:space="preserve">  "content": [{</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "q_answer": ["1. ", "2. ", "3. ", "4. "],</t>
+          <t xml:space="preserve">    "q_text": "사람들이 무엇을 하고 있습니까?",</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "q_correct": 2</t>
+          <t xml:space="preserve">    "q_image_description": {</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  }]</t>
+          <t xml:space="preserve">      "image": "여자가 부엌에서 빨래를 하고 있다. 세탁기 옆에 빨래 바구니가 있다."</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">    },</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "q_answer": ["1. ", "2. ", "3. ", "4. "],</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "q_correct": 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  }]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
           <t>}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="38">
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A66:F66"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A27:F27"/>
     <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A50:F50"/>
     <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A55:F55"/>
     <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A42:F42"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="A17:F17"/>
@@ -5385,26 +5496,26 @@
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A62:F62"/>
     <mergeCell ref="A53:F53"/>
-    <mergeCell ref="A29:F29"/>
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A63:F63"/>
-    <mergeCell ref="A52:F52"/>
-    <mergeCell ref="A65:F65"/>
-    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="A67:F67"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A58:F58"/>
     <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A40:F40"/>
     <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A39:F39"/>
     <mergeCell ref="A64:F64"/>
     <mergeCell ref="A59:F59"/>
     <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A49:F49"/>
-    <mergeCell ref="A51:F51"/>
     <mergeCell ref="A60:F60"/>
     <mergeCell ref="A36:F36"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A70:F70"/>
     <mergeCell ref="A61:F61"/>
-    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A69:F69"/>
+    <mergeCell ref="A65:F65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5416,7 +5527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5670,252 +5781,314 @@
       <c r="F24" s="10" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>Không phát hiện bẫy rõ — đáp án dựa trên hình ảnh.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Bẫy</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Tỷ lệ</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Mô tả</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>`trap_action_swap`</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Bức sai có đúng bối cảnh nhưng sai hành động</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>`trap_context_swap`</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Bức sai có đúng hành động nhưng sai bối cảnh/nơi chốn</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>`trap_detail_distort`</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Bức sai đúng tổng thể nhưng sai chi tiết nhỏ</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Cấu trúc audio</t>
         </is>
       </c>
-      <c r="B26" s="10" t="n"/>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
-      <c r="E26" s="10" t="n"/>
-      <c r="F26" s="10" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>• Hội thoại ngắn giữa 가/나 (2-3 lượt nói), nội dung về hoạt động hàng ngày</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>• Format: 가: 몇 시에 일어납니까?\n나: 여섯 시에 일어납니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Cấu trúc đáp án</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="n"/>
-      <c r="C29" s="10" t="n"/>
-      <c r="D29" s="10" t="n"/>
-      <c r="E29" s="10" t="n"/>
-      <c r="F29" s="10" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>• q_answer: ["①", "②", "③", "④"] (310003) hoặc ["1", "2", "3", "4"] (3410006)</t>
-        </is>
-      </c>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>• q_text: rỗng</t>
+          <t>• Hội thoại ngắn giữa 가/나 (2-3 lượt nói), nội dung về hoạt động hàng ngày</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>• q_image: có (4 ảnh mỗi câu)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t>• 4 bức tranh minh họa các cảnh khác nhau → dùng q_image_description để mô tả</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>Cách mô tả ảnh (q_image_description)</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="10" t="n"/>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
+          <t>• Format: 가: 몇 시에 일어납니까?\n나: 여섯 시에 일어납니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
+        <is>
+          <t>Cấu trúc đáp án</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="n"/>
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="10" t="n"/>
+      <c r="E33" s="10" t="n"/>
+      <c r="F33" s="10" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>• q_answer: ["①", "②", "③", "④"] (310003) hoặc ["1", "2", "3", "4"] (3410006)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>Mỗi bức tranh mô tả một cảnh sinh hoạt. Mô tả bao gồm: ai đang làm gì, ở đâu, chi tiết quan trọng phân biệt các bức.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>Quy tắc tạo 4 bức tranh</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="n"/>
-      <c r="C36" s="10" t="n"/>
-      <c r="D36" s="10" t="n"/>
-      <c r="E36" s="10" t="n"/>
-      <c r="F36" s="10" t="n"/>
+          <t>• q_text: rỗng</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>• q_image: có (4 ảnh mỗi câu)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
-          <t>• Bức đúng: khớp chính xác nội dung audio (hành động + bối cảnh + đối tượng)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>• Bức sai 1: đúng bối cảnh nhưng sai hành động</t>
-        </is>
-      </c>
+          <t>• 4 bức tranh minh họa các cảnh khác nhau → dùng q_image_description để mô tả</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Cách mô tả ảnh (q_image_description)</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
+          <t>Mỗi bức tranh mô tả một cảnh sinh hoạt. Mô tả bao gồm: ai đang làm gì, ở đâu, chi tiết quan trọng phân biệt các bức.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Quy tắc tạo 4 bức tranh</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="n"/>
+      <c r="C40" s="10" t="n"/>
+      <c r="D40" s="10" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>• Bức đúng: khớp chính xác nội dung audio (hành động + bối cảnh + đối tượng)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>• Bức sai 1: đúng bối cảnh nhưng sai hành động</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
           <t>• Bức sai 2: đúng hành động nhưng sai bối cảnh</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t>• Bức sai 3: khác hoàn toàn nhưng dùng 1 yếu tố gây nhầm lẫn từ audio</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="9" t="inlineStr">
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>Ví dụ</t>
         </is>
       </c>
-      <c r="B41" s="10" t="n"/>
-      <c r="C41" s="10" t="n"/>
-      <c r="D41" s="10" t="n"/>
-      <c r="E41" s="10" t="n"/>
-      <c r="F41" s="10" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="12" t="inlineStr">
-        <is>
-          <t>{</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  "g_text_audio": "가: 몇 시에 일어납니까?\n나: 여섯 시에 일어납니다.",</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  "content": [{</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    "q_image_description": {</t>
-        </is>
-      </c>
+      <c r="B45" s="10" t="n"/>
+      <c r="C45" s="10" t="n"/>
+      <c r="D45" s="10" t="n"/>
+      <c r="E45" s="10" t="n"/>
+      <c r="F45" s="10" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "1": "남자가 아침 6시에 침대에서 일어나고 있다. 알람시계가 6:00을 가리킨다.",</t>
+          <t>{</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "2": "남자가 밤에 침대에 누워 자고 있다. 시계가 10:00을 가리킨다.",</t>
+          <t xml:space="preserve">  "g_text_audio": "가: 몇 시에 일어납니까?\n나: 여섯 시에 일어납니다.",</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "3": "남자가 아침에 운동을 하고 있다. 공원에서 조깅.",</t>
+          <t xml:space="preserve">  "content": [{</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">      "4": "남자가 아침 식사를 하고 있다. 식탁에 앉아 있다."</t>
+          <t xml:space="preserve">    "q_image_description": {</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    },</t>
+          <t xml:space="preserve">      "1": "남자가 아침 6시에 침대에서 일어나고 있다. 알람시계가 6:00을 가리킨다.",</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "q_answer": ["①", "②", "③", "④"],</t>
+          <t xml:space="preserve">      "2": "남자가 밤에 침대에 누워 자고 있다. 시계가 10:00을 가리킨다.",</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    "q_correct": 1</t>
+          <t xml:space="preserve">      "3": "남자가 아침에 운동을 하고 있다. 공원에서 조깅.",</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  }]</t>
+          <t xml:space="preserve">      "4": "남자가 아침 식사를 하고 있다. 식탁에 앉아 있다."</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">    },</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "q_answer": ["①", "②", "③", "④"],</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    "q_correct": 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  }]</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="inlineStr">
+        <is>
           <t>}</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="37">
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A27:F27"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A50:F50"/>
-    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A56:F56"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A57:F57"/>
     <mergeCell ref="A33:F33"/>
     <mergeCell ref="A47:F47"/>
     <mergeCell ref="A42:F42"/>
@@ -5925,13 +6098,12 @@
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A53:F53"/>
-    <mergeCell ref="A29:F29"/>
     <mergeCell ref="A43:F43"/>
     <mergeCell ref="A38:F38"/>
     <mergeCell ref="A52:F52"/>
-    <mergeCell ref="A28:F28"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A58:F58"/>
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="A48:F48"/>
@@ -5943,7 +6115,6 @@
     <mergeCell ref="A36:F36"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A45:F45"/>
-    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>